<commit_message>
Daily NSE scan: 2026-10-08
</commit_message>
<xml_diff>
--- a/output/2026-10-08/enriched_analysis.xlsx
+++ b/output/2026-10-08/enriched_analysis.xlsx
@@ -929,10 +929,10 @@
         </is>
       </c>
       <c r="V2" t="n">
-        <v>2.062</v>
+        <v>2.067</v>
       </c>
       <c r="W2" t="n">
-        <v>3055</v>
+        <v>3048</v>
       </c>
       <c r="X2" t="n">
         <v>23.9</v>
@@ -1396,7 +1396,7 @@
         <v>0.045</v>
       </c>
       <c r="W4" t="n">
-        <v>2926</v>
+        <v>2929</v>
       </c>
       <c r="X4" t="n">
         <v>10.1</v>
@@ -1855,13 +1855,13 @@
         </is>
       </c>
       <c r="V6" t="n">
-        <v>1.195</v>
+        <v>1.177</v>
       </c>
       <c r="W6" t="n">
-        <v>314</v>
+        <v>319</v>
       </c>
       <c r="X6" t="n">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="Y6" t="n">
         <v>22</v>
@@ -2090,7 +2090,7 @@
         <v>0.325</v>
       </c>
       <c r="W7" t="n">
-        <v>942</v>
+        <v>943</v>
       </c>
       <c r="X7" t="n">
         <v>9.27</v>
@@ -2319,13 +2319,13 @@
         </is>
       </c>
       <c r="V8" t="n">
-        <v>1.127</v>
+        <v>1.115</v>
       </c>
       <c r="W8" t="n">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="X8" t="n">
-        <v>7.57</v>
+        <v>7.66</v>
       </c>
       <c r="Y8" t="n">
         <v>17</v>
@@ -2551,13 +2551,13 @@
         </is>
       </c>
       <c r="V9" t="n">
-        <v>0.538</v>
+        <v>0.537</v>
       </c>
       <c r="W9" t="n">
-        <v>2654</v>
+        <v>2659</v>
       </c>
       <c r="X9" t="n">
-        <v>21.7</v>
+        <v>21.8</v>
       </c>
       <c r="Y9" t="n">
         <v>8</v>
@@ -2786,7 +2786,7 @@
         <v>0.048</v>
       </c>
       <c r="W10" t="n">
-        <v>14926</v>
+        <v>14929</v>
       </c>
       <c r="X10" t="n">
         <v>38</v>
@@ -3015,13 +3015,13 @@
         </is>
       </c>
       <c r="V11" t="n">
-        <v>2.275</v>
+        <v>2.272</v>
       </c>
       <c r="W11" t="n">
-        <v>2580</v>
+        <v>2583</v>
       </c>
       <c r="X11" t="n">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="Y11" t="n">
         <v>6</v>
@@ -3250,7 +3250,7 @@
         <v>0.05</v>
       </c>
       <c r="W12" t="n">
-        <v>1651</v>
+        <v>1648</v>
       </c>
       <c r="X12" t="n">
         <v>22.2</v>
@@ -3479,13 +3479,13 @@
         </is>
       </c>
       <c r="V13" t="n">
-        <v>0.063</v>
+        <v>0.064</v>
       </c>
       <c r="W13" t="n">
-        <v>893</v>
+        <v>885</v>
       </c>
       <c r="X13" t="n">
-        <v>22.6</v>
+        <v>22.4</v>
       </c>
       <c r="Y13" t="n">
         <v>19</v>
@@ -3712,7 +3712,7 @@
         <v>0.125</v>
       </c>
       <c r="W14" t="n">
-        <v>2510</v>
+        <v>2506</v>
       </c>
       <c r="X14" t="n">
         <v>22</v>
@@ -3944,10 +3944,10 @@
         <v>0.065</v>
       </c>
       <c r="W15" t="n">
-        <v>1708</v>
+        <v>1713</v>
       </c>
       <c r="X15" t="n">
-        <v>39.2</v>
+        <v>39.3</v>
       </c>
       <c r="Y15" t="n">
         <v>20</v>
@@ -4173,10 +4173,10 @@
         </is>
       </c>
       <c r="V16" t="n">
-        <v>2.815</v>
+        <v>2.811</v>
       </c>
       <c r="W16" t="n">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="X16" t="n">
         <v>21.1</v>
@@ -4629,13 +4629,13 @@
         </is>
       </c>
       <c r="V18" t="n">
-        <v>0.189</v>
+        <v>0.179</v>
       </c>
       <c r="W18" t="n">
-        <v>586</v>
+        <v>618</v>
       </c>
       <c r="X18" t="n">
-        <v>49</v>
+        <v>51.6</v>
       </c>
       <c r="Y18" t="n">
         <v>3</v>
@@ -4867,7 +4867,7 @@
         <v>834</v>
       </c>
       <c r="X19" t="n">
-        <v>36.3</v>
+        <v>36.4</v>
       </c>
       <c r="Y19" t="n">
         <v>17</v>
@@ -5090,10 +5090,10 @@
         <v>0.089</v>
       </c>
       <c r="W20" t="n">
-        <v>642</v>
+        <v>639</v>
       </c>
       <c r="X20" t="n">
-        <v>10.5</v>
+        <v>10.4</v>
       </c>
       <c r="Y20" t="n">
         <v>-5</v>
@@ -5319,13 +5319,13 @@
         </is>
       </c>
       <c r="V21" t="n">
-        <v>0.37</v>
+        <v>0.375</v>
       </c>
       <c r="W21" t="n">
-        <v>1064</v>
+        <v>1049</v>
       </c>
       <c r="X21" t="n">
-        <v>54.2</v>
+        <v>53.5</v>
       </c>
       <c r="Y21" t="n">
         <v>21</v>
@@ -5554,7 +5554,7 @@
         <v>0.008999999999999999</v>
       </c>
       <c r="W22" t="n">
-        <v>54142</v>
+        <v>54091</v>
       </c>
       <c r="X22" t="n">
         <v>45.8</v>
@@ -5789,7 +5789,7 @@
         <v>435</v>
       </c>
       <c r="X23" t="n">
-        <v>10.9</v>
+        <v>10.8</v>
       </c>
       <c r="Y23" t="n">
         <v>19</v>
@@ -5943,12 +5943,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>SRGHFL</t>
+          <t>STUDDS</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>SRG HOUSING FINANCE LIMITED</t>
+          <t>Studds Accessories Limited</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -5960,40 +5960,40 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="F24" t="n">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="G24" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H24" t="n">
         <v>0</v>
       </c>
       <c r="I24" t="n">
-        <v>126.61</v>
+        <v>420.45</v>
       </c>
       <c r="J24" t="n">
-        <v>132.2</v>
+        <v>417.34</v>
       </c>
       <c r="K24" t="n">
-        <v>-4.2</v>
+        <v>0.7</v>
       </c>
       <c r="L24" t="n">
-        <v>67.83</v>
+        <v>61.75</v>
       </c>
       <c r="M24" t="n">
-        <v>1.98</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="N24" t="n">
-        <v>19830410</v>
+        <v>6931636</v>
       </c>
       <c r="O24" t="n">
         <v>0</v>
       </c>
       <c r="P24" t="n">
-        <v>19830410</v>
+        <v>6931636</v>
       </c>
       <c r="Q24" t="n">
         <v>0</v>
@@ -6007,56 +6007,60 @@
         <v>0</v>
       </c>
       <c r="T24" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="U24" t="inlineStr">
         <is>
-          <t>16-09-2026</t>
+          <t>11-09-2026</t>
         </is>
       </c>
       <c r="V24" t="n">
-        <v>1.002</v>
+        <v>0.042</v>
       </c>
       <c r="W24" t="n">
-        <v>198</v>
+        <v>1655</v>
       </c>
       <c r="X24" t="n">
-        <v>5.8</v>
+        <v>21.6</v>
       </c>
       <c r="Y24" t="n">
-        <v>31</v>
-      </c>
-      <c r="Z24" t="inlineStr"/>
+        <v>10</v>
+      </c>
+      <c r="Z24" t="n">
+        <v>20</v>
+      </c>
       <c r="AA24" t="n">
-        <v>35</v>
+        <v>2</v>
       </c>
       <c r="AB24" t="n">
-        <v>5.39</v>
+        <v>3.37</v>
       </c>
       <c r="AC24" t="n">
-        <v>11.8</v>
+        <v>23.3</v>
       </c>
       <c r="AD24" t="n">
-        <v>2.89</v>
+        <v>0.01</v>
       </c>
       <c r="AE24" t="b">
-        <v>0</v>
-      </c>
-      <c r="AF24" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="AF24" t="n">
+        <v>12</v>
+      </c>
       <c r="AG24" t="n">
-        <v>222.99</v>
+        <v>428.24</v>
       </c>
       <c r="AH24" t="n">
-        <v>265.05</v>
+        <v>474.36</v>
       </c>
       <c r="AI24" t="n">
-        <v>-48.6</v>
+        <v>-5.5</v>
       </c>
       <c r="AJ24" t="n">
-        <v>132.2027333333333</v>
+        <v>417.3421638870492</v>
       </c>
       <c r="AK24" t="n">
-        <v>-4.2</v>
+        <v>0.7</v>
       </c>
       <c r="AL24" t="inlineStr">
         <is>
@@ -6065,47 +6069,47 @@
       </c>
       <c r="AM24" t="inlineStr">
         <is>
+          <t>Mature Accumulation</t>
+        </is>
+      </c>
+      <c r="AN24" t="inlineStr">
+        <is>
           <t>Confirmed Accumulation</t>
         </is>
       </c>
-      <c r="AN24" t="inlineStr">
-        <is>
-          <t>Confirmed Accumulation</t>
-        </is>
-      </c>
       <c r="AO24" t="inlineStr">
         <is>
-          <t>15-09-2026</t>
+          <t>11-09-2026</t>
         </is>
       </c>
       <c r="AP24" t="inlineStr">
         <is>
-          <t>16-09-2026</t>
+          <t>11-09-2026</t>
         </is>
       </c>
       <c r="AQ24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR24" t="n">
+        <v>27</v>
+      </c>
+      <c r="AS24" t="n">
+        <v>27</v>
+      </c>
+      <c r="AT24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV24" t="n">
         <v>1</v>
       </c>
-      <c r="AR24" t="n">
-        <v>23</v>
-      </c>
-      <c r="AS24" t="n">
-        <v>22</v>
-      </c>
-      <c r="AT24" t="n">
-        <v>0</v>
-      </c>
-      <c r="AU24" t="n">
-        <v>0</v>
-      </c>
-      <c r="AV24" t="n">
-        <v>3</v>
-      </c>
       <c r="AW24" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AX24" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AY24" t="n">
         <v>0</v>
@@ -6114,13 +6118,13 @@
         <v>0</v>
       </c>
       <c r="BA24" t="n">
-        <v>19830410</v>
+        <v>6931636</v>
       </c>
       <c r="BB24" t="n">
-        <v>19830410</v>
+        <v>6931636</v>
       </c>
       <c r="BC24" t="n">
-        <v>19830410</v>
+        <v>6931636</v>
       </c>
       <c r="BD24" t="n">
         <v>0</v>
@@ -6156,10 +6160,10 @@
         <v>0</v>
       </c>
       <c r="BO24" t="n">
-        <v>19830410</v>
+        <v>6931636</v>
       </c>
       <c r="BP24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="BQ24" t="n">
         <v>0</v>
@@ -6171,12 +6175,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>STUDDS</t>
+          <t>TAINWALCHM</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Studds Accessories Limited</t>
+          <t>TAINWALA CHEMICALS AND PLASTICS (INDIA) LIMITED</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -6188,171 +6192,171 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="F25" t="n">
+        <v>6</v>
+      </c>
+      <c r="G25" t="n">
+        <v>13</v>
+      </c>
+      <c r="H25" t="n">
+        <v>-1</v>
+      </c>
+      <c r="I25" t="n">
+        <v>200.4</v>
+      </c>
+      <c r="J25" t="n">
+        <v>210.19</v>
+      </c>
+      <c r="K25" t="n">
+        <v>-4.7</v>
+      </c>
+      <c r="L25" t="n">
+        <v>67.04000000000001</v>
+      </c>
+      <c r="M25" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="N25" t="n">
+        <v>6171564</v>
+      </c>
+      <c r="O25" t="n">
+        <v>0</v>
+      </c>
+      <c r="P25" t="n">
+        <v>6171564</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>0</v>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>Net Buying</t>
+        </is>
+      </c>
+      <c r="S25" t="b">
+        <v>0</v>
+      </c>
+      <c r="T25" t="n">
+        <v>14</v>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>28-09-2026</t>
+        </is>
+      </c>
+      <c r="V25" t="n">
+        <v>0.328</v>
+      </c>
+      <c r="W25" t="n">
+        <v>188</v>
+      </c>
+      <c r="X25" t="n">
+        <v>23.3</v>
+      </c>
+      <c r="Y25" t="n">
+        <v>12</v>
+      </c>
+      <c r="Z25" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="AA25" t="n">
         <v>16</v>
       </c>
-      <c r="G25" t="n">
-        <v>4</v>
-      </c>
-      <c r="H25" t="n">
-        <v>0</v>
-      </c>
-      <c r="I25" t="n">
-        <v>420.45</v>
-      </c>
-      <c r="J25" t="n">
-        <v>417.34</v>
-      </c>
-      <c r="K25" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="L25" t="n">
-        <v>61.75</v>
-      </c>
-      <c r="M25" t="n">
-        <v>0.6899999999999999</v>
-      </c>
-      <c r="N25" t="n">
-        <v>6931636</v>
-      </c>
-      <c r="O25" t="n">
-        <v>0</v>
-      </c>
-      <c r="P25" t="n">
-        <v>6931636</v>
-      </c>
-      <c r="Q25" t="n">
-        <v>0</v>
-      </c>
-      <c r="R25" t="inlineStr">
-        <is>
-          <t>Net Buying</t>
-        </is>
-      </c>
-      <c r="S25" t="b">
-        <v>0</v>
-      </c>
-      <c r="T25" t="n">
+      <c r="AB25" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="AC25" t="n">
+        <v>7.91</v>
+      </c>
+      <c r="AD25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE25" t="b">
+        <v>0</v>
+      </c>
+      <c r="AF25" t="n">
+        <v>3.16</v>
+      </c>
+      <c r="AG25" t="n">
+        <v>208.91</v>
+      </c>
+      <c r="AH25" t="n">
+        <v>197.78</v>
+      </c>
+      <c r="AI25" t="n">
+        <v>12.1</v>
+      </c>
+      <c r="AJ25" t="n">
+        <v>210.188815475785</v>
+      </c>
+      <c r="AK25" t="n">
+        <v>-4.7</v>
+      </c>
+      <c r="AL25" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="AM25" t="inlineStr">
+        <is>
+          <t>Confirmed Accumulation</t>
+        </is>
+      </c>
+      <c r="AN25" t="inlineStr">
+        <is>
+          <t>Confirmed Accumulation</t>
+        </is>
+      </c>
+      <c r="AO25" t="inlineStr">
+        <is>
+          <t>18-08-2026</t>
+        </is>
+      </c>
+      <c r="AP25" t="inlineStr">
+        <is>
+          <t>28-09-2026</t>
+        </is>
+      </c>
+      <c r="AQ25" t="n">
+        <v>41</v>
+      </c>
+      <c r="AR25" t="n">
+        <v>51</v>
+      </c>
+      <c r="AS25" t="n">
+        <v>10</v>
+      </c>
+      <c r="AT25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU25" t="n">
         <v>1</v>
       </c>
-      <c r="U25" t="inlineStr">
-        <is>
-          <t>11-09-2026</t>
-        </is>
-      </c>
-      <c r="V25" t="n">
-        <v>0.042</v>
-      </c>
-      <c r="W25" t="n">
-        <v>1656</v>
-      </c>
-      <c r="X25" t="n">
-        <v>21.6</v>
-      </c>
-      <c r="Y25" t="n">
-        <v>10</v>
-      </c>
-      <c r="Z25" t="n">
-        <v>20</v>
-      </c>
-      <c r="AA25" t="n">
-        <v>2</v>
-      </c>
-      <c r="AB25" t="n">
-        <v>3.37</v>
-      </c>
-      <c r="AC25" t="n">
-        <v>23.3</v>
-      </c>
-      <c r="AD25" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="AE25" t="b">
-        <v>1</v>
-      </c>
-      <c r="AF25" t="n">
-        <v>12</v>
-      </c>
-      <c r="AG25" t="n">
-        <v>428.24</v>
-      </c>
-      <c r="AH25" t="n">
-        <v>474.36</v>
-      </c>
-      <c r="AI25" t="n">
-        <v>-5.5</v>
-      </c>
-      <c r="AJ25" t="n">
-        <v>417.3421638870492</v>
-      </c>
-      <c r="AK25" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="AL25" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="AM25" t="inlineStr">
-        <is>
-          <t>Mature Accumulation</t>
-        </is>
-      </c>
-      <c r="AN25" t="inlineStr">
-        <is>
-          <t>Confirmed Accumulation</t>
-        </is>
-      </c>
-      <c r="AO25" t="inlineStr">
-        <is>
-          <t>11-09-2026</t>
-        </is>
-      </c>
-      <c r="AP25" t="inlineStr">
-        <is>
-          <t>11-09-2026</t>
-        </is>
-      </c>
-      <c r="AQ25" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR25" t="n">
-        <v>27</v>
-      </c>
-      <c r="AS25" t="n">
-        <v>27</v>
-      </c>
-      <c r="AT25" t="n">
-        <v>0</v>
-      </c>
-      <c r="AU25" t="n">
-        <v>0</v>
-      </c>
       <c r="AV25" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="AW25" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="AX25" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="AY25" t="n">
         <v>0</v>
       </c>
       <c r="AZ25" t="n">
-        <v>0</v>
+        <v>131838</v>
       </c>
       <c r="BA25" t="n">
-        <v>6931636</v>
+        <v>3024580</v>
       </c>
       <c r="BB25" t="n">
-        <v>6931636</v>
+        <v>6171564</v>
       </c>
       <c r="BC25" t="n">
-        <v>6931636</v>
+        <v>6171564</v>
       </c>
       <c r="BD25" t="n">
         <v>0</v>
@@ -6388,7 +6392,7 @@
         <v>0</v>
       </c>
       <c r="BO25" t="n">
-        <v>6931636</v>
+        <v>3024580</v>
       </c>
       <c r="BP25" t="n">
         <v>1</v>
@@ -6403,16 +6407,16 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>TAINWALCHM</t>
+          <t>SINCLAIR</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>TAINWALA CHEMICALS AND PLASTICS (INDIA) LIMITED</t>
+          <t>SINCLAIRS HOTELS LIMITED</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -6420,40 +6424,40 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="F26" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G26" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="H26" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="I26" t="n">
-        <v>200.4</v>
+        <v>75.09999999999999</v>
       </c>
       <c r="J26" t="n">
-        <v>210.19</v>
+        <v>81.09999999999999</v>
       </c>
       <c r="K26" t="n">
-        <v>-4.7</v>
+        <v>-7.4</v>
       </c>
       <c r="L26" t="n">
-        <v>67.04000000000001</v>
+        <v>62.78</v>
       </c>
       <c r="M26" t="n">
-        <v>0.62</v>
+        <v>2</v>
       </c>
       <c r="N26" t="n">
-        <v>6171564</v>
+        <v>19959718</v>
       </c>
       <c r="O26" t="n">
         <v>0</v>
       </c>
       <c r="P26" t="n">
-        <v>6171564</v>
+        <v>19959718</v>
       </c>
       <c r="Q26" t="n">
         <v>0</v>
@@ -6467,94 +6471,94 @@
         <v>0</v>
       </c>
       <c r="T26" t="n">
+        <v>8</v>
+      </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>24-09-2026</t>
+        </is>
+      </c>
+      <c r="V26" t="n">
+        <v>0.518</v>
+      </c>
+      <c r="W26" t="n">
+        <v>385</v>
+      </c>
+      <c r="X26" t="n">
+        <v>35.7</v>
+      </c>
+      <c r="Y26" t="n">
+        <v>21</v>
+      </c>
+      <c r="Z26" t="n">
+        <v>8.390000000000001</v>
+      </c>
+      <c r="AA26" t="n">
+        <v>-19</v>
+      </c>
+      <c r="AB26" t="n">
+        <v>1.54</v>
+      </c>
+      <c r="AC26" t="n">
+        <v>8.73</v>
+      </c>
+      <c r="AD26" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="AE26" t="b">
+        <v>1</v>
+      </c>
+      <c r="AF26" t="n">
+        <v>41.64</v>
+      </c>
+      <c r="AG26" t="n">
+        <v>78.06</v>
+      </c>
+      <c r="AH26" t="n">
+        <v>77.62</v>
+      </c>
+      <c r="AI26" t="n">
+        <v>-1.9</v>
+      </c>
+      <c r="AJ26" t="n">
+        <v>81.10277768748172</v>
+      </c>
+      <c r="AK26" t="n">
+        <v>-7.4</v>
+      </c>
+      <c r="AL26" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="AM26" t="inlineStr">
+        <is>
+          <t>Confirmed Accumulation</t>
+        </is>
+      </c>
+      <c r="AN26" t="inlineStr">
+        <is>
+          <t>Confirmed Accumulation</t>
+        </is>
+      </c>
+      <c r="AO26" t="inlineStr">
+        <is>
+          <t>28-08-2026</t>
+        </is>
+      </c>
+      <c r="AP26" t="inlineStr">
+        <is>
+          <t>24-09-2026</t>
+        </is>
+      </c>
+      <c r="AQ26" t="n">
+        <v>27</v>
+      </c>
+      <c r="AR26" t="n">
+        <v>41</v>
+      </c>
+      <c r="AS26" t="n">
         <v>14</v>
-      </c>
-      <c r="U26" t="inlineStr">
-        <is>
-          <t>28-09-2026</t>
-        </is>
-      </c>
-      <c r="V26" t="n">
-        <v>0.323</v>
-      </c>
-      <c r="W26" t="n">
-        <v>191</v>
-      </c>
-      <c r="X26" t="n">
-        <v>23.7</v>
-      </c>
-      <c r="Y26" t="n">
-        <v>12</v>
-      </c>
-      <c r="Z26" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="AA26" t="n">
-        <v>16</v>
-      </c>
-      <c r="AB26" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="AC26" t="n">
-        <v>7.91</v>
-      </c>
-      <c r="AD26" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE26" t="b">
-        <v>0</v>
-      </c>
-      <c r="AF26" t="n">
-        <v>3.16</v>
-      </c>
-      <c r="AG26" t="n">
-        <v>208.91</v>
-      </c>
-      <c r="AH26" t="n">
-        <v>197.78</v>
-      </c>
-      <c r="AI26" t="n">
-        <v>12.1</v>
-      </c>
-      <c r="AJ26" t="n">
-        <v>210.188815475785</v>
-      </c>
-      <c r="AK26" t="n">
-        <v>-4.7</v>
-      </c>
-      <c r="AL26" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="AM26" t="inlineStr">
-        <is>
-          <t>Confirmed Accumulation</t>
-        </is>
-      </c>
-      <c r="AN26" t="inlineStr">
-        <is>
-          <t>Confirmed Accumulation</t>
-        </is>
-      </c>
-      <c r="AO26" t="inlineStr">
-        <is>
-          <t>18-08-2026</t>
-        </is>
-      </c>
-      <c r="AP26" t="inlineStr">
-        <is>
-          <t>28-09-2026</t>
-        </is>
-      </c>
-      <c r="AQ26" t="n">
-        <v>41</v>
-      </c>
-      <c r="AR26" t="n">
-        <v>51</v>
-      </c>
-      <c r="AS26" t="n">
-        <v>10</v>
       </c>
       <c r="AT26" t="n">
         <v>0</v>
@@ -6563,28 +6567,28 @@
         <v>1</v>
       </c>
       <c r="AV26" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="AW26" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="AX26" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="AY26" t="n">
         <v>0</v>
       </c>
       <c r="AZ26" t="n">
-        <v>131838</v>
+        <v>1417187</v>
       </c>
       <c r="BA26" t="n">
-        <v>3024580</v>
+        <v>3357558</v>
       </c>
       <c r="BB26" t="n">
-        <v>6171564</v>
+        <v>19959718</v>
       </c>
       <c r="BC26" t="n">
-        <v>6171564</v>
+        <v>19959718</v>
       </c>
       <c r="BD26" t="n">
         <v>0</v>
@@ -6620,7 +6624,7 @@
         <v>0</v>
       </c>
       <c r="BO26" t="n">
-        <v>3024580</v>
+        <v>3357558</v>
       </c>
       <c r="BP26" t="n">
         <v>1</v>
@@ -6635,12 +6639,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>SINCLAIR</t>
+          <t>SRGHFL</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>SINCLAIRS HOTELS LIMITED</t>
+          <t>SRG HOUSING FINANCE LIMITED</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -6652,40 +6656,40 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F27" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G27" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H27" t="n">
         <v>0</v>
       </c>
       <c r="I27" t="n">
-        <v>75.09999999999999</v>
+        <v>126.61</v>
       </c>
       <c r="J27" t="n">
-        <v>81.09999999999999</v>
+        <v>132.2</v>
       </c>
       <c r="K27" t="n">
-        <v>-7.4</v>
+        <v>-4.2</v>
       </c>
       <c r="L27" t="n">
-        <v>62.78</v>
+        <v>67.83</v>
       </c>
       <c r="M27" t="n">
-        <v>2</v>
+        <v>1.98</v>
       </c>
       <c r="N27" t="n">
-        <v>19959718</v>
+        <v>19830410</v>
       </c>
       <c r="O27" t="n">
         <v>0</v>
       </c>
       <c r="P27" t="n">
-        <v>19959718</v>
+        <v>19830410</v>
       </c>
       <c r="Q27" t="n">
         <v>0</v>
@@ -6699,124 +6703,120 @@
         <v>0</v>
       </c>
       <c r="T27" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="U27" t="inlineStr">
         <is>
-          <t>24-09-2026</t>
+          <t>16-09-2026</t>
         </is>
       </c>
       <c r="V27" t="n">
-        <v>0.516</v>
+        <v>0.997</v>
       </c>
       <c r="W27" t="n">
-        <v>387</v>
+        <v>199</v>
       </c>
       <c r="X27" t="n">
-        <v>35.9</v>
+        <v>5.82</v>
       </c>
       <c r="Y27" t="n">
-        <v>21</v>
-      </c>
-      <c r="Z27" t="n">
-        <v>8.390000000000001</v>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="Z27" t="inlineStr"/>
       <c r="AA27" t="n">
-        <v>-19</v>
+        <v>35</v>
       </c>
       <c r="AB27" t="n">
-        <v>1.54</v>
+        <v>5.39</v>
       </c>
       <c r="AC27" t="n">
-        <v>8.73</v>
+        <v>11.8</v>
       </c>
       <c r="AD27" t="n">
-        <v>0.28</v>
+        <v>2.89</v>
       </c>
       <c r="AE27" t="b">
+        <v>0</v>
+      </c>
+      <c r="AF27" t="inlineStr"/>
+      <c r="AG27" t="n">
+        <v>222.99</v>
+      </c>
+      <c r="AH27" t="n">
+        <v>265.05</v>
+      </c>
+      <c r="AI27" t="n">
+        <v>-48.6</v>
+      </c>
+      <c r="AJ27" t="n">
+        <v>132.2027333333333</v>
+      </c>
+      <c r="AK27" t="n">
+        <v>-4.2</v>
+      </c>
+      <c r="AL27" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="AM27" t="inlineStr">
+        <is>
+          <t>Confirmed Accumulation</t>
+        </is>
+      </c>
+      <c r="AN27" t="inlineStr">
+        <is>
+          <t>Confirmed Accumulation</t>
+        </is>
+      </c>
+      <c r="AO27" t="inlineStr">
+        <is>
+          <t>15-09-2026</t>
+        </is>
+      </c>
+      <c r="AP27" t="inlineStr">
+        <is>
+          <t>16-09-2026</t>
+        </is>
+      </c>
+      <c r="AQ27" t="n">
         <v>1</v>
       </c>
-      <c r="AF27" t="n">
-        <v>41.64</v>
-      </c>
-      <c r="AG27" t="n">
-        <v>78.06</v>
-      </c>
-      <c r="AH27" t="n">
-        <v>77.62</v>
-      </c>
-      <c r="AI27" t="n">
-        <v>-1.9</v>
-      </c>
-      <c r="AJ27" t="n">
-        <v>81.10277768748172</v>
-      </c>
-      <c r="AK27" t="n">
-        <v>-7.4</v>
-      </c>
-      <c r="AL27" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="AM27" t="inlineStr">
-        <is>
-          <t>Confirmed Accumulation</t>
-        </is>
-      </c>
-      <c r="AN27" t="inlineStr">
-        <is>
-          <t>Confirmed Accumulation</t>
-        </is>
-      </c>
-      <c r="AO27" t="inlineStr">
-        <is>
-          <t>28-08-2026</t>
-        </is>
-      </c>
-      <c r="AP27" t="inlineStr">
-        <is>
-          <t>24-09-2026</t>
-        </is>
-      </c>
-      <c r="AQ27" t="n">
-        <v>27</v>
-      </c>
       <c r="AR27" t="n">
-        <v>41</v>
+        <v>23</v>
       </c>
       <c r="AS27" t="n">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="AT27" t="n">
         <v>0</v>
       </c>
       <c r="AU27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AV27" t="n">
         <v>3</v>
       </c>
       <c r="AW27" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="AX27" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="AY27" t="n">
         <v>0</v>
       </c>
       <c r="AZ27" t="n">
-        <v>1417187</v>
+        <v>0</v>
       </c>
       <c r="BA27" t="n">
-        <v>3357558</v>
+        <v>19830410</v>
       </c>
       <c r="BB27" t="n">
-        <v>19959718</v>
+        <v>19830410</v>
       </c>
       <c r="BC27" t="n">
-        <v>19959718</v>
+        <v>19830410</v>
       </c>
       <c r="BD27" t="n">
         <v>0</v>
@@ -6852,10 +6852,10 @@
         <v>0</v>
       </c>
       <c r="BO27" t="n">
-        <v>3357558</v>
+        <v>19830410</v>
       </c>
       <c r="BP27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BQ27" t="n">
         <v>0</v>
@@ -6939,13 +6939,13 @@
         </is>
       </c>
       <c r="V28" t="n">
-        <v>0.516</v>
+        <v>0.514</v>
       </c>
       <c r="W28" t="n">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="X28" t="n">
-        <v>36</v>
+        <v>36.3</v>
       </c>
       <c r="Y28" t="n">
         <v>-44</v>
@@ -7629,13 +7629,13 @@
         </is>
       </c>
       <c r="V31" t="n">
-        <v>0.277</v>
+        <v>0.276</v>
       </c>
       <c r="W31" t="n">
-        <v>941</v>
+        <v>943</v>
       </c>
       <c r="X31" t="n">
-        <v>25.6</v>
+        <v>25.7</v>
       </c>
       <c r="Y31" t="n">
         <v>9</v>
@@ -7861,13 +7861,13 @@
         </is>
       </c>
       <c r="V32" t="n">
-        <v>0.645</v>
+        <v>0.65</v>
       </c>
       <c r="W32" t="n">
-        <v>364</v>
+        <v>361</v>
       </c>
       <c r="X32" t="n">
-        <v>1174</v>
+        <v>1165</v>
       </c>
       <c r="Y32" t="n">
         <v>-61</v>
@@ -8089,13 +8089,13 @@
         </is>
       </c>
       <c r="V33" t="n">
-        <v>0.239</v>
+        <v>0.234</v>
       </c>
       <c r="W33" t="n">
-        <v>271</v>
+        <v>277</v>
       </c>
       <c r="X33" t="n">
-        <v>14.3</v>
+        <v>14.6</v>
       </c>
       <c r="Y33" t="n">
         <v>16</v>
@@ -8324,7 +8324,7 @@
         <v>0.821</v>
       </c>
       <c r="W34" t="n">
-        <v>3847</v>
+        <v>3849</v>
       </c>
       <c r="X34" t="n">
         <v>26.9</v>
@@ -8556,7 +8556,7 @@
         <v>0.232</v>
       </c>
       <c r="W35" t="n">
-        <v>1722</v>
+        <v>1721</v>
       </c>
       <c r="X35" t="n">
         <v>18.2</v>
@@ -9017,13 +9017,13 @@
         </is>
       </c>
       <c r="V37" t="n">
-        <v>0.361</v>
+        <v>0.363</v>
       </c>
       <c r="W37" t="n">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="X37" t="n">
-        <v>95.90000000000001</v>
+        <v>95.5</v>
       </c>
       <c r="Y37" t="n">
         <v>246</v>
@@ -9252,7 +9252,7 @@
         <v>0</v>
       </c>
       <c r="W38" t="n">
-        <v>5507</v>
+        <v>5511</v>
       </c>
       <c r="X38" t="n">
         <v>12.9</v>
@@ -9484,10 +9484,10 @@
         <v>0.114</v>
       </c>
       <c r="W39" t="n">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="X39" t="n">
-        <v>7.02</v>
+        <v>7.04</v>
       </c>
       <c r="Y39" t="n">
         <v>118</v>
@@ -9712,7 +9712,7 @@
         <v>0.011</v>
       </c>
       <c r="W40" t="n">
-        <v>4135</v>
+        <v>4125</v>
       </c>
       <c r="X40" t="inlineStr"/>
       <c r="Y40" t="n">
@@ -10174,7 +10174,7 @@
         <v>0.076</v>
       </c>
       <c r="W42" t="n">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="X42" t="n">
         <v>13.1</v>
@@ -10406,10 +10406,10 @@
         <v>0.101</v>
       </c>
       <c r="W43" t="n">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="X43" t="n">
-        <v>27.1</v>
+        <v>27.2</v>
       </c>
       <c r="Y43" t="n">
         <v>24</v>
@@ -10635,10 +10635,10 @@
         </is>
       </c>
       <c r="V44" t="n">
-        <v>0.053</v>
+        <v>0.052</v>
       </c>
       <c r="W44" t="n">
-        <v>932</v>
+        <v>940</v>
       </c>
       <c r="X44" t="inlineStr"/>
       <c r="Y44" t="n">
@@ -10868,10 +10868,10 @@
         <v>0</v>
       </c>
       <c r="W45" t="n">
-        <v>3873</v>
+        <v>3870</v>
       </c>
       <c r="X45" t="n">
-        <v>87.2</v>
+        <v>87.09999999999999</v>
       </c>
       <c r="Y45" t="n">
         <v>42</v>
@@ -11100,10 +11100,10 @@
         <v>0.006</v>
       </c>
       <c r="W46" t="n">
-        <v>4901</v>
+        <v>4904</v>
       </c>
       <c r="X46" t="n">
-        <v>12.6</v>
+        <v>12.7</v>
       </c>
       <c r="Y46" t="n">
         <v>23</v>
@@ -11328,7 +11328,7 @@
         <v>0</v>
       </c>
       <c r="W47" t="n">
-        <v>108321</v>
+        <v>108231</v>
       </c>
       <c r="X47" t="n">
         <v>31.2</v>
@@ -11557,13 +11557,13 @@
         </is>
       </c>
       <c r="V48" t="n">
-        <v>0.219</v>
+        <v>0.221</v>
       </c>
       <c r="W48" t="n">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="X48" t="n">
-        <v>24.4</v>
+        <v>24.1</v>
       </c>
       <c r="Y48" t="n">
         <v>21</v>
@@ -12559,140 +12559,140 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>SRGHFL</t>
+          <t>STUDDS</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>SRG HOUSING FINANCE LIMITED</t>
+          <t>Studds Accessories Limited</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>126.61</v>
+        <v>420.45</v>
       </c>
       <c r="D24" t="n">
-        <v>132.2</v>
+        <v>417.34</v>
       </c>
       <c r="E24" t="n">
-        <v>-4.2</v>
+        <v>0.7</v>
       </c>
       <c r="F24" t="n">
-        <v>67.83</v>
+        <v>61.75</v>
       </c>
       <c r="G24" t="n">
-        <v>1.98</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="H24" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>16-09-2026</t>
+          <t>11-09-2026</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>STUDDS</t>
+          <t>TAINWALCHM</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Studds Accessories Limited</t>
+          <t>TAINWALA CHEMICALS AND PLASTICS (INDIA) LIMITED</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>420.45</v>
+        <v>200.4</v>
       </c>
       <c r="D25" t="n">
-        <v>417.34</v>
+        <v>210.19</v>
       </c>
       <c r="E25" t="n">
-        <v>0.7</v>
+        <v>-4.7</v>
       </c>
       <c r="F25" t="n">
-        <v>61.75</v>
+        <v>67.04000000000001</v>
       </c>
       <c r="G25" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.62</v>
       </c>
       <c r="H25" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>11-09-2026</t>
+          <t>28-09-2026</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>TAINWALCHM</t>
+          <t>SINCLAIR</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>TAINWALA CHEMICALS AND PLASTICS (INDIA) LIMITED</t>
+          <t>SINCLAIRS HOTELS LIMITED</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>200.4</v>
+        <v>75.09999999999999</v>
       </c>
       <c r="D26" t="n">
-        <v>210.19</v>
+        <v>81.09999999999999</v>
       </c>
       <c r="E26" t="n">
-        <v>-4.7</v>
+        <v>-7.4</v>
       </c>
       <c r="F26" t="n">
-        <v>67.04000000000001</v>
+        <v>62.78</v>
       </c>
       <c r="G26" t="n">
-        <v>0.62</v>
+        <v>2</v>
       </c>
       <c r="H26" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>28-09-2026</t>
+          <t>24-09-2026</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>SINCLAIR</t>
+          <t>SRGHFL</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>SINCLAIRS HOTELS LIMITED</t>
+          <t>SRG HOUSING FINANCE LIMITED</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>75.09999999999999</v>
+        <v>126.61</v>
       </c>
       <c r="D27" t="n">
-        <v>81.09999999999999</v>
+        <v>132.2</v>
       </c>
       <c r="E27" t="n">
-        <v>-7.4</v>
+        <v>-4.2</v>
       </c>
       <c r="F27" t="n">
-        <v>62.78</v>
+        <v>67.83</v>
       </c>
       <c r="G27" t="n">
-        <v>2</v>
+        <v>1.98</v>
       </c>
       <c r="H27" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>24-09-2026</t>
+          <t>16-09-2026</t>
         </is>
       </c>
     </row>

</xml_diff>